<commit_message>
Knocked all of leftover debt: 20 tasks from critical to wbns. Going to audit and test now before progressing with next steps.
Update .gitignore and CHANGELOG; enhance database connection management and logging

- Updated .gitignore to include .venv/ for virtual environment exclusion.
- Added a PEP 561 marker to CHANGELOG.md to ensure type information is recognized by type checkers.
- Refactored database connection handling in cli.py and db.py to use context managers for better resource management.
- Introduced logging configuration in cli.py to enable debug logging via command-line options.
- Improved the handling of database connections in various CLI commands to ensure proper cleanup and avoid leaks.
</commit_message>
<xml_diff>
--- a/tests/fixtures/empty.xlsx
+++ b/tests/fixtures/empty.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Empty" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empty" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Working on the 2nd half (obvs)  - missing audit and retros + reviews but implementation sort of completed:
new benchmarking features and observability enhancements

- Added a new section in CHANGELOG.md for schema version 2.0, detailing the introduction of the `hermes bench` command for benchmarking workloads, including memory and performance metrics.
- Expanded README.md to include comprehensive instructions on running benchmarks, including command usage, flags, and methodology for measuring performance and memory usage.
- Updated the evaluation and health metrics roadmap to reflect the completion of observability tasks, including structured logging and RSS sampling.
- Documented the migration from version 1.0 to 2.0 of the observability schema, clarifying changes in stage names and logging behavior.
</commit_message>
<xml_diff>
--- a/tests/fixtures/empty.xlsx
+++ b/tests/fixtures/empty.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empty" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Empty" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Completed eval + healt and quant:
Enhance evaluation framework and observability features

- Added a new section in CHANGELOG.md for schema version 2.0, detailing updates to the evaluation subsystem, including anchor-based record matching and page-range resolution.
- Updated README.md to include instructions on using the new `field_type_hint` and `match_key` features for scoring, along with clarifications on how to interpret evaluation results.
- Expanded configuration options in config.toml.example to support observability features, including logging format and RSS sampling settings.
- Documented changes in the evaluation and health metrics roadmap, reflecting the completion of major audit findings and enhancements to the evaluation framework.
- Introduced new decision logs and packets for T8 and T9 tasks, detailing the architectural decisions made for anchor-based matching and page-range resolution.
</commit_message>
<xml_diff>
--- a/tests/fixtures/empty.xlsx
+++ b/tests/fixtures/empty.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Empty" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empty" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>